<commit_message>
Add optionlet and swaption volatility
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_volatilities.xlsx
+++ b/tests/workbooks/test_volatilities.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{856D44B6-9674-459E-947D-D4C724D76103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5645EFE-9191-4203-A449-172AEF82A6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2460" yWindow="-17900" windowWidth="23040" windowHeight="14790" xr2:uid="{03D12B07-F690-4065-A8E3-371E349FECFA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{03D12B07-F690-4065-A8E3-371E349FECFA}"/>
   </bookViews>
   <sheets>
     <sheet name="qlBlackConstantVol" sheetId="1" r:id="rId1"/>
+    <sheet name="qlConstantOptionletVolatility" sheetId="2" r:id="rId2"/>
+    <sheet name="qlConstantSwaptionVolatility" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="63">
   <si>
     <t>Reference date</t>
   </si>
@@ -130,16 +132,163 @@
   </si>
   <si>
     <t>qlBlackVolTermStructureBlackForwardVarianceFromTime</t>
+  </si>
+  <si>
+    <t>reference_date</t>
+  </si>
+  <si>
+    <t>Reference date for the volatility.,</t>
+  </si>
+  <si>
+    <t>calendar</t>
+  </si>
+  <si>
+    <t>Calendar for the volatility.,</t>
+  </si>
+  <si>
+    <t>business_day_convention</t>
+  </si>
+  <si>
+    <t>Business day convention for the volatility.,</t>
+  </si>
+  <si>
+    <t>volatility</t>
+  </si>
+  <si>
+    <t>Constant volatility value.,</t>
+  </si>
+  <si>
+    <t>day_counter</t>
+  </si>
+  <si>
+    <t>Day count convention for the volatility.,</t>
+  </si>
+  <si>
+    <t>volatility_type</t>
+  </si>
+  <si>
+    <t>Volatility type (e.g. 'NORMAL', 'SHIFTEDLOGNORMAL').,</t>
+  </si>
+  <si>
+    <t>shift</t>
+  </si>
+  <si>
+    <t>Shift value for shifted lognormal volatility.,</t>
+  </si>
+  <si>
+    <t>Following</t>
+  </si>
+  <si>
+    <t>qlConstantOptionletVolatility</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>expiry_date</t>
+  </si>
+  <si>
+    <t>strike</t>
+  </si>
+  <si>
+    <t>extrapolate</t>
+  </si>
+  <si>
+    <t>qlOptionletVolatilityStructureVolatility</t>
+  </si>
+  <si>
+    <t>qlOptionletVolatilityStructureVolatilityFromTime</t>
+  </si>
+  <si>
+    <t>qlOptionletVolatilityStructureBlackVariance</t>
+  </si>
+  <si>
+    <t>qlOptionletVolatilityStructureBlackVarianceFromTime</t>
+  </si>
+  <si>
+    <t>qlConstantSwaptionVolatility</t>
+  </si>
+  <si>
+    <t>swap_tenor</t>
+  </si>
+  <si>
+    <t>2y</t>
+  </si>
+  <si>
+    <t>swap_length</t>
+  </si>
+  <si>
+    <t>expiry_term</t>
+  </si>
+  <si>
+    <t>1y</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureOptionDateFromTenor</t>
+  </si>
+  <si>
+    <t>qlTermStructureTimeFromReference</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureVolatility</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureVolatilityFromTime</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureBlackVariance</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureBlackVarianceFromTime</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureShift</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureShiftFromTime</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureSmileSection</t>
+  </si>
+  <si>
+    <t>qlSwaptionVolatilityStructureSmileSectionFromTime</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0000%"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -162,16 +311,43 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -548,7 +724,7 @@
       </c>
       <c r="B6" t="str" cm="1">
         <f t="array" ref="B6">_xll.qlBlackConstantVol(B1,B2,B3,B4)</f>
-        <v>⚡[test_volatilities.xlsx]qlBlackConstantVol!R6C2BlackVolTermStructureHandle,A</v>
+        <v>欣[test_volatilities.xlsx]qlBlackConstantVol!R6C2BlackVolTermStructureHandle,A</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -693,6 +869,524 @@
       <c r="B28" cm="1">
         <f t="array" ref="B28">_xll.qlBlackVolTermStructureBlackForwardVarianceFromTime(B6,B12,B16,B13)</f>
         <v>6.25E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2E334E1-BB58-4274-97F9-2A66D842EB70}">
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="44.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4">
+        <v>46174</v>
+      </c>
+      <c r="C1" s="4">
+        <v>46174</v>
+      </c>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="C4" s="7">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="3" t="str" cm="1">
+        <f t="array" ref="B8">_xll.qlConstantOptionletVolatility(B1,B2,B3,B4,B5)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantOptionletVolatility!R8C2OptionletVolatilityStructureHandle,A</v>
+      </c>
+      <c r="C8" s="3" t="str" cm="1">
+        <f t="array" ref="C8">_xll.qlConstantOptionletVolatility(C1,C2,C3,C4,C5,C6,C7)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantOptionletVolatility!R8C3OptionletVolatilityStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="4">
+        <f>B1+365</f>
+        <v>46539</v>
+      </c>
+      <c r="C10" s="4">
+        <f>C1+365</f>
+        <v>46539</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="9" cm="1">
+        <f t="array" ref="B11">_xll.qlTermStructureTimeFromReference(B8,B10)</f>
+        <v>1</v>
+      </c>
+      <c r="C11" s="9" cm="1">
+        <f t="array" ref="C11">_xll.qlTermStructureTimeFromReference(C8,C10)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="6" cm="1">
+        <f t="array" ref="B15">_xll.qlOptionletVolatilityStructureVolatility(B8,B10,B12)</f>
+        <v>0.25</v>
+      </c>
+      <c r="C15" s="7" cm="1">
+        <f t="array" ref="C15">_xll.qlOptionletVolatilityStructureVolatility(C8,C10,C12,C13)</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="6" cm="1">
+        <f t="array" ref="B16">_xll.qlOptionletVolatilityStructureVolatilityFromTime(B8,B11,B12)</f>
+        <v>0.25</v>
+      </c>
+      <c r="C16" s="7" cm="1">
+        <f t="array" ref="C16">_xll.qlOptionletVolatilityStructureVolatilityFromTime(C8,C11,C12,C13)</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="7" cm="1">
+        <f t="array" ref="B17">_xll.qlOptionletVolatilityStructureBlackVariance(B8,B10,B12)</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C17" s="10" cm="1">
+        <f t="array" ref="C17">_xll.qlOptionletVolatilityStructureBlackVariance(C8,C10,C12,C13)</f>
+        <v>6.3999999999999997E-5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="7" cm="1">
+        <f t="array" ref="B18">_xll.qlOptionletVolatilityStructureBlackVarianceFromTime(B8,B11,B12)</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C18" s="10" cm="1">
+        <f t="array" ref="C18">_xll.qlOptionletVolatilityStructureBlackVarianceFromTime(C8,C11,C12,C13)</f>
+        <v>6.3999999999999997E-5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F7DD04-F97D-41C9-B20D-15577F3B15F2}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="44.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="32.21875" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4">
+        <v>46174</v>
+      </c>
+      <c r="C1" s="4">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="C4" s="7">
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="3" t="str" cm="1">
+        <f t="array" ref="B8">_xll.qlConstantSwaptionVolatility(B1,B2,B3,B4,B5)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantSwaptionVolatility!R8C2SwaptionVolatilityStructureHandle,A</v>
+      </c>
+      <c r="C8" s="3" t="str" cm="1">
+        <f t="array" ref="C8">_xll.qlConstantSwaptionVolatility(C1,C2,C3,C4,C5,C6,C7)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantSwaptionVolatility!R8C3SwaptionVolatilityStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="4" cm="1">
+        <f t="array" ref="B11">_xll.qlSwaptionVolatilityStructureOptionDateFromTenor(B8,B10)</f>
+        <v>46539</v>
+      </c>
+      <c r="C11" s="4" cm="1">
+        <f t="array" ref="C11">_xll.qlSwaptionVolatilityStructureOptionDateFromTenor(C8,C10)</f>
+        <v>46539</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="9" cm="1">
+        <f t="array" ref="B12">_xll.qlTermStructureTimeFromReference(B8,B11)</f>
+        <v>1</v>
+      </c>
+      <c r="C12" s="9" cm="1">
+        <f t="array" ref="C12">_xll.qlTermStructureTimeFromReference(C8,C11)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="8">
+        <v>2</v>
+      </c>
+      <c r="C14" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="6" cm="1">
+        <f t="array" ref="B18">_xll.qlSwaptionVolatilityStructureVolatility(B8,B11,B13,B15)</f>
+        <v>0.25</v>
+      </c>
+      <c r="C18" s="7" cm="1">
+        <f t="array" ref="C18">_xll.qlSwaptionVolatilityStructureVolatility(C8,C11,C13,C15,C16)</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="6" cm="1">
+        <f t="array" ref="B19">_xll.qlSwaptionVolatilityStructureVolatilityFromTime(B8,B12,B14,B15)</f>
+        <v>0.25</v>
+      </c>
+      <c r="C19" s="7" cm="1">
+        <f t="array" ref="C19">_xll.qlSwaptionVolatilityStructureVolatilityFromTime(C8,C12,C14,C15,C16)</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" s="7" cm="1">
+        <f t="array" ref="B20">_xll.qlSwaptionVolatilityStructureBlackVariance(B8,B11,B13,B15)</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C20" s="10" cm="1">
+        <f t="array" ref="C20">_xll.qlSwaptionVolatilityStructureBlackVariance(C8,C11,C13,C15,C16)</f>
+        <v>6.3999999999999997E-5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="7" cm="1">
+        <f t="array" ref="B21">_xll.qlSwaptionVolatilityStructureBlackVarianceFromTime(B8,B12,B14,B15)</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C21" s="10" cm="1">
+        <f t="array" ref="C21">_xll.qlSwaptionVolatilityStructureBlackVarianceFromTime(C8,C12,C14,C15)</f>
+        <v>6.3999999999999997E-5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="7" cm="1">
+        <f t="array" ref="B22">_xll.qlSwaptionVolatilityStructureShift(B8,B11,B13)</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="11" t="str" cm="1">
+        <f t="array" ref="C22">_xll.qlSwaptionVolatilityStructureShift(C8,C11,C13,C16)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: shift parameter only makes sense for lognormal volatilities
+Traceback (most recent call last):
+  File "C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\src\quantlib_xloil\volatilities.py", line 760, in qlSwaptionVolatilityStructureShift
+    return vol_tsh.shift(option_date, swap_tenor, extrapolate)
+           ~~~~~~~~~~~~~^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+  File "C:\Users\Sebastian\.conda\envs\xloil\Lib\site-packages\QuantLib\QuantLib.py", line 12304, in shift
+    return _QuantLib.SwaptionVolatilityStructureHandle_shift(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: shift parameter only makes sense for lognormal volatilities
+</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="7" cm="1">
+        <f t="array" ref="B23">_xll.qlSwaptionVolatilityStructureShiftFromTime(B8,B12,B14)</f>
+        <v>0</v>
+      </c>
+      <c r="C23" s="11" t="str" cm="1">
+        <f t="array" ref="C23">_xll.qlSwaptionVolatilityStructureShiftFromTime(C8,C12,C14,C16)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: shift parameter only makes sense for lognormal volatilities
+Traceback (most recent call last):
+  File "C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\src\quantlib_xloil\volatilities.py", line 781, in qlSwaptionVolatilityStructureShiftFromTime
+    return vol_tsh.shift(option_time, swap_length, extrapolate)
+           ~~~~~~~~~~~~~^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+  File "C:\Users\Sebastian\.conda\envs\xloil\Lib\site-packages\QuantLib\QuantLib.py", line 12304, in shift
+    return _QuantLib.SwaptionVolatilityStructureHandle_shift(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: shift parameter only makes sense for lognormal volatilities
+</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="3" t="str" cm="1">
+        <f t="array" ref="B24">_xll.qlSwaptionVolatilityStructureSmileSection(B8,B11,B13)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantSwaptionVolatility!R24C2SmileSection,A</v>
+      </c>
+      <c r="C24" s="3" t="str" cm="1">
+        <f t="array" ref="C24">_xll.qlSwaptionVolatilityStructureSmileSection(C8,C11,C13,C16)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantSwaptionVolatility!R24C3SmileSection,C</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="3" t="str" cm="1">
+        <f t="array" ref="B25">_xll.qlSwaptionVolatilityStructureSmileSectionFromTime(B8,B12,B14)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantSwaptionVolatility!R25C2SmileSection,A</v>
+      </c>
+      <c r="C25" s="3" t="str" cm="1">
+        <f t="array" ref="C25">_xll.qlSwaptionVolatilityStructureSmileSectionFromTime(C8,C12,C14,C16)</f>
+        <v>欣[test_volatilities.xlsx]qlConstantSwaptionVolatility!R25C3SmileSection,A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>